<commit_message>
Updates to employee portal, attendance portal, and login page
</commit_message>
<xml_diff>
--- a/attendance/python-script/all_users_main_branch.xlsx
+++ b/attendance/python-script/all_users_main_branch.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1384"/>
+  <dimension ref="A1:E1416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37784,6 +37784,870 @@
         </is>
       </c>
     </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>1384</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>Rahimakhan</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>1385</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>Hussainalikhan</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>1386</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>Sherazali</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>1387</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>Muneeb</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>1388</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>Tariqjamil</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>1389</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>Farrukhmir</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>1390</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>Khateja</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>1391</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>Sufiyanahmed</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>1392</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>Mwaize</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>1393</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>Huzaifa</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>1394</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>Abdullah</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>1395</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>Murtaza</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>1396</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>Hassam</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>1397</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>Liaqatullah</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>1398</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>Umerzahid</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>1399</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>Umerali</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1400" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>Ahmad</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>1401</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>Mohsin</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>1402</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>Mantasha</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>1403</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>Muneeb</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1404" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr">
+        <is>
+          <t>1404</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>Hamzatariq</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1405" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1405" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr">
+        <is>
+          <t>1405</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>Abdulmuneam</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1406" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1406" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr">
+        <is>
+          <t>1406</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>Sahil</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1407" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1407" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr">
+        <is>
+          <t>1407</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>Ahtisham</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1408" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1408" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr">
+        <is>
+          <t>1408</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>Bilal</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1409" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1409" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr">
+        <is>
+          <t>1409</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>Waleed</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1410" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1410" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr">
+        <is>
+          <t>1410</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>Saqibali</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1411" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1411" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr">
+        <is>
+          <t>1411</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>Mhammad</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1412" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1412" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr">
+        <is>
+          <t>1412</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>hassan</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1413" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1413" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr">
+        <is>
+          <t>1413</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>Wajahat</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1414" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1414" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr">
+        <is>
+          <t>1414</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>Shahmeer</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1415" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1415" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr">
+        <is>
+          <t>1415</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>Arooj</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="D1416" t="inlineStr">
+        <is>
+          <t>Main Branch</t>
+        </is>
+      </c>
+      <c r="E1416" t="inlineStr">
+        <is>
+          <t>203.215.161.244</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>